<commit_message>
Actualizo predicciones dado que se juega ATA-COM suspendido ayer.
</commit_message>
<xml_diff>
--- a/data/italy/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
+++ b/data/italy/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,10 +461,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>id_player_miss_home_4</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>player_name_miss_home_4</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>id_player_miss_away_1</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>player_name_miss_away_1</t>
         </is>
@@ -478,344 +488,54 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>nD7QhgLn</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>godfrey ben</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>hvC4gron</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>scalvini giorgio</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>vDgQxOYl</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>scamacca gianluca</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>QB1RMomj</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>toloi rafael</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>t20vQIvC</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>varane raphael</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>CCDxBZAc</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>pIgDNCf3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>KIQjmWIj</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Whh3dzd4</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>WxCQa92d</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>OC8I1VXq</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>h8tCfEQG</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>0YqKhheT</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>WETw9DuA</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>vuXo7iAM</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>z3jsi9f5</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>8SWavWAa</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>WUqjkmPH</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>EB8yv2aJ</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>ttV7xAuC</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>x8OGzlAO</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>dzYLoEIP</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>SW3Qfiet</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>lnhZhVPh</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>SIOithtm</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>